<commit_message>
Preserve draft edits and complete cache pricing imports
</commit_message>
<xml_diff>
--- a/artifacts/mortgage-budget.xlsx
+++ b/artifacts/mortgage-budget.xlsx
@@ -2065,7 +2065,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>51e97dbd-04ab-4159-b857-07079c0bd83b</t>
+          <t>3a025782-4666-472c-a542-34ef1803f2ce</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2092,7 +2092,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>f8c40808-98cf-4159-a6d6-7761a0f0444c</t>
+          <t>42a064ea-b8ab-4b07-8147-f9a9b14e2075</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2225,7 +2225,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-09-23T19:39:08.578Z</t>
+          <t>2026-09-25T21:24:19.328Z</t>
         </is>
       </c>
       <c r="I2" s="2" t="b">

</xml_diff>